<commit_message>
feat:ultimos cambios antes de empaquetado
</commit_message>
<xml_diff>
--- a/apps/web/public/formato_clientes.xlsx
+++ b/apps/web/public/formato_clientes.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="35">
   <si>
     <t>RUC</t>
   </si>
@@ -31,7 +31,7 @@
     <t>Condicion por defecto</t>
   </si>
   <si>
-    <t>Medio de pago por defecto</t>
+    <t>Código de pago por defecto</t>
   </si>
   <si>
     <t>IGV por defecto</t>
@@ -47,22 +47,88 @@
   </si>
   <si>
     <t>Cuenta de Compras</t>
+  </si>
+  <si>
+    <t>20123456789</t>
+  </si>
+  <si>
+    <t>EMPRESA UNO S.A.C.</t>
+  </si>
+  <si>
+    <t>EMP UNO</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>CLIENTE LOCAL</t>
+  </si>
+  <si>
+    <t>CONTADO</t>
+  </si>
+  <si>
+    <t>TRANSFERENCIA</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>500.00</t>
+  </si>
+  <si>
+    <t>SI</t>
+  </si>
+  <si>
+    <t>121201</t>
+  </si>
+  <si>
+    <t>421201</t>
+  </si>
+  <si>
+    <t>10442962893</t>
+  </si>
+  <si>
+    <t>ALARCON PRETELL ANGEL ALEXANDER</t>
+  </si>
+  <si>
+    <t>ALARCON ANGEL</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>PERSONA NATURAL</t>
+  </si>
+  <si>
+    <t>CREDITO 15 DIAS</t>
+  </si>
+  <si>
+    <t>YAPE</t>
+  </si>
+  <si>
+    <t>300.00</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>121202</t>
+  </si>
+  <si>
+    <t>421202</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
       <scheme val="minor"/>
       <sz val="11"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
     </font>
   </fonts>
   <fills count="2">
@@ -85,9 +151,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -427,57 +492,133 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="4" width="20" customWidth="1"/>
+    <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="25" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="25" customWidth="1"/>
-    <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="9" width="20" customWidth="1"/>
-    <col min="10" max="10" width="15" customWidth="1"/>
+    <col min="6" max="7" width="25" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="25" customWidth="1"/>
+    <col min="10" max="10" width="18" customWidth="1"/>
     <col min="11" max="12" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K2" t="s">
+        <v>22</v>
+      </c>
+      <c r="L2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G3" t="s">
+        <v>30</v>
+      </c>
+      <c r="H3" t="s">
+        <v>19</v>
+      </c>
+      <c r="I3" t="s">
+        <v>31</v>
+      </c>
+      <c r="J3" t="s">
+        <v>32</v>
+      </c>
+      <c r="K3" t="s">
+        <v>33</v>
+      </c>
+      <c r="L3" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Release v0.1.4: Fix excel mapping and template
</commit_message>
<xml_diff>
--- a/apps/web/public/formato_clientes.xlsx
+++ b/apps/web/public/formato_clientes.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>RUC</t>
   </si>
@@ -43,92 +43,38 @@
     <t>Declara PLAME</t>
   </si>
   <si>
+    <t>Declara AFPNET</t>
+  </si>
+  <si>
+    <t>Declara ITAN</t>
+  </si>
+  <si>
+    <t>Declara DAOT</t>
+  </si>
+  <si>
+    <t>Declara PDT 710</t>
+  </si>
+  <si>
     <t>Cuenta de Ventas</t>
   </si>
   <si>
     <t>Cuenta de Compras</t>
-  </si>
-  <si>
-    <t>20123456789</t>
-  </si>
-  <si>
-    <t>EMPRESA UNO S.A.C.</t>
-  </si>
-  <si>
-    <t>EMP UNO</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>CLIENTE LOCAL</t>
-  </si>
-  <si>
-    <t>CONTADO</t>
-  </si>
-  <si>
-    <t>TRANSFERENCIA</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>500.00</t>
-  </si>
-  <si>
-    <t>SI</t>
-  </si>
-  <si>
-    <t>121201</t>
-  </si>
-  <si>
-    <t>421201</t>
-  </si>
-  <si>
-    <t>10442962893</t>
-  </si>
-  <si>
-    <t>ALARCON PRETELL ANGEL ALEXANDER</t>
-  </si>
-  <si>
-    <t>ALARCON ANGEL</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>PERSONA NATURAL</t>
-  </si>
-  <si>
-    <t>CREDITO 15 DIAS</t>
-  </si>
-  <si>
-    <t>YAPE</t>
-  </si>
-  <si>
-    <t>300.00</t>
-  </si>
-  <si>
-    <t>NO</t>
-  </si>
-  <si>
-    <t>121202</t>
-  </si>
-  <si>
-    <t>421202</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
       <scheme val="minor"/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
     </font>
   </fonts>
   <fills count="2">
@@ -151,8 +97,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -492,133 +439,69 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="40" customWidth="1"/>
-    <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="25" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="4" width="20" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="7" width="25" customWidth="1"/>
-    <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="25" customWidth="1"/>
-    <col min="10" max="10" width="18" customWidth="1"/>
-    <col min="11" max="12" width="20" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="7" max="7" width="25" customWidth="1"/>
+    <col min="8" max="8" width="15" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="10" max="14" width="15" customWidth="1"/>
+    <col min="15" max="16" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B2" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C2" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D2" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="E2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H2" t="s">
-        <v>19</v>
-      </c>
-      <c r="I2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" t="s">
-        <v>21</v>
-      </c>
-      <c r="K2" t="s">
-        <v>22</v>
-      </c>
-      <c r="L2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G3" t="s">
-        <v>30</v>
-      </c>
-      <c r="H3" t="s">
-        <v>19</v>
-      </c>
-      <c r="I3" t="s">
-        <v>31</v>
-      </c>
-      <c r="J3" t="s">
-        <v>32</v>
-      </c>
-      <c r="K3" t="s">
-        <v>33</v>
-      </c>
-      <c r="L3" t="s">
-        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Release v0.1.5: Fix client accounts mapping
</commit_message>
<xml_diff>
--- a/apps/web/public/formato_clientes.xlsx
+++ b/apps/web/public/formato_clientes.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>RUC</t>
   </si>
@@ -46,19 +46,28 @@
     <t>Declara AFPNET</t>
   </si>
   <si>
+    <t>Declara Benif. Final</t>
+  </si>
+  <si>
     <t>Declara ITAN</t>
   </si>
   <si>
     <t>Declara DAOT</t>
   </si>
   <si>
-    <t>Declara PDT 710</t>
-  </si>
-  <si>
-    <t>Cuenta de Ventas</t>
-  </si>
-  <si>
-    <t>Cuenta de Compras</t>
+    <t>Declara PDT 710 Anual</t>
+  </si>
+  <si>
+    <t>Cuenta de Ventas Base</t>
+  </si>
+  <si>
+    <t>Cuenta Venta total</t>
+  </si>
+  <si>
+    <t>Cuenta de Compras Base</t>
+  </si>
+  <si>
+    <t>Cuenta Compra total</t>
   </si>
 </sst>
 </file>
@@ -439,7 +448,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:S1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -450,11 +459,17 @@
     <col min="7" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
     <col min="9" max="9" width="20" customWidth="1"/>
-    <col min="10" max="14" width="15" customWidth="1"/>
-    <col min="15" max="16" width="20" customWidth="1"/>
+    <col min="10" max="11" width="15" customWidth="1"/>
+    <col min="12" max="12" width="20" customWidth="1"/>
+    <col min="13" max="14" width="15" customWidth="1"/>
+    <col min="15" max="15" width="20" customWidth="1"/>
+    <col min="16" max="16" width="25" customWidth="1"/>
+    <col min="17" max="17" width="20" customWidth="1"/>
+    <col min="18" max="18" width="25" customWidth="1"/>
+    <col min="19" max="19" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -502,6 +517,15 @@
       </c>
       <c r="P1" s="1" t="s">
         <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>